<commit_message>
Novedades del período: días, licencias, descuentos y LRE real
Separa ficha permanente de novedades mensuales (ausencias, licencia,
feriado, horas extras, bonos y descuentos con tipo). Proporcionaliza
sueldo/colación/movilización, valida art. 58, bloquea líquido negativo
y emite LRE 1115/1116/1117/3188 desde datos reales.

Co-authored-by: kco_ai <Cryptobal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ejemplos/trabajadores.xlsx
+++ b/ejemplos/trabajadores.xlsx
@@ -58,75 +58,80 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t xml:space="preserve">fecha_termino</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t xml:space="preserve">jornada</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t xml:space="preserve">horas_extras</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t xml:space="preserve">colacion</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t xml:space="preserve">movilizacion</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">gratificacion</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t xml:space="preserve">email</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t xml:space="preserve">banco</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t xml:space="preserve">tipo_cuenta</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t xml:space="preserve">nro_cuenta</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_nombre</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_monto</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_imponible</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_nombre</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_monto</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_imponible</t>
         </is>
@@ -178,77 +183,77 @@
           <t xml:space="preserve">01/03/2023</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t xml:space="preserve">50000</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">40000</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t xml:space="preserve">ana@empresa.cl</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t xml:space="preserve">001</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t xml:space="preserve">corriente</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t xml:space="preserve">12345678</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono producción</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t xml:space="preserve">80000</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t xml:space="preserve">Colación extra</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t xml:space="preserve">15000</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
@@ -300,77 +305,77 @@
           <t xml:space="preserve">15/01/2025</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t xml:space="preserve">8</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t xml:space="preserve">40000</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">35000</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t xml:space="preserve">luis@empresa.cl</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t xml:space="preserve">012</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t xml:space="preserve">vista</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t xml:space="preserve">11111111</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono asistencia</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t xml:space="preserve">30000</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t xml:space="preserve">Movilización extra</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t xml:space="preserve">12000</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
@@ -422,77 +427,77 @@
           <t xml:space="preserve">01/06/2022</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t xml:space="preserve">60000</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">50000</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t xml:space="preserve">camila@empresa.cl</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t xml:space="preserve">037</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t xml:space="preserve">corriente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t xml:space="preserve">98765432</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono de cargo</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t xml:space="preserve">90000</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t xml:space="preserve">Asignación de movilización</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t xml:space="preserve">20000</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>

</xml_diff>

<commit_message>
Novedades del período: días, licencias, descuentos y LRE real (#20)
Separa ficha permanente de novedades mensuales (ausencias, licencia,
feriado, horas extras, bonos y descuentos con tipo). Proporcionaliza
sueldo/colación/movilización, valida art. 58, bloquea líquido negativo
y emite LRE 1115/1116/1117/3188 desde datos reales.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: kco_ai <Cryptobal@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ejemplos/trabajadores.xlsx
+++ b/ejemplos/trabajadores.xlsx
@@ -58,75 +58,80 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t xml:space="preserve">fecha_termino</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t xml:space="preserve">jornada</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t xml:space="preserve">horas_extras</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t xml:space="preserve">colacion</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t xml:space="preserve">movilizacion</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">gratificacion</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t xml:space="preserve">email</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t xml:space="preserve">banco</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t xml:space="preserve">tipo_cuenta</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t xml:space="preserve">nro_cuenta</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_nombre</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_monto</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_1_imponible</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_nombre</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_monto</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t xml:space="preserve">bono_2_imponible</t>
         </is>
@@ -178,77 +183,77 @@
           <t xml:space="preserve">01/03/2023</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t xml:space="preserve">50000</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">40000</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t xml:space="preserve">ana@empresa.cl</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t xml:space="preserve">001</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t xml:space="preserve">corriente</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t xml:space="preserve">12345678</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono producción</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t xml:space="preserve">80000</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t xml:space="preserve">Colación extra</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t xml:space="preserve">15000</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
@@ -300,77 +305,77 @@
           <t xml:space="preserve">15/01/2025</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t xml:space="preserve">8</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t xml:space="preserve">40000</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">35000</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t xml:space="preserve">luis@empresa.cl</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t xml:space="preserve">012</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t xml:space="preserve">vista</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t xml:space="preserve">11111111</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono asistencia</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t xml:space="preserve">30000</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t xml:space="preserve">Movilización extra</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t xml:space="preserve">12000</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>
@@ -422,77 +427,77 @@
           <t xml:space="preserve">01/06/2022</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">42</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t xml:space="preserve">60000</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">50000</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t xml:space="preserve">camila@empresa.cl</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t xml:space="preserve">037</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t xml:space="preserve">corriente</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t xml:space="preserve">98765432</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t xml:space="preserve">Bono de cargo</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t xml:space="preserve">90000</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t xml:space="preserve">si</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t xml:space="preserve">Asignación de movilización</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t xml:space="preserve">20000</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t xml:space="preserve">no</t>
         </is>

</xml_diff>